<commit_message>
fix: implement `Meter`/`Yard` user input to customer order
it's a conversion for DR printing option
</commit_message>
<xml_diff>
--- a/Report Files/DeliveryReceipt/DeliveryReceiptExcel.xlsx
+++ b/Report Files/DeliveryReceipt/DeliveryReceiptExcel.xlsx
@@ -334,54 +334,69 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="B6:C47"/>
+  <dimension ref="B1:D47"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="4" max="4" width="55.42578125" customWidth="1"/>
+    <col min="4" max="4" width="55.42578125" style="1" customWidth="1"/>
     <col min="5" max="5" width="12.42578125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="6" spans="2:3" x14ac:dyDescent="0.25">
+    <row r="1" spans="2:4" x14ac:dyDescent="0.25">
+      <c r="D1"/>
+    </row>
+    <row r="2" spans="2:4" x14ac:dyDescent="0.25">
+      <c r="D2"/>
+    </row>
+    <row r="3" spans="2:4" x14ac:dyDescent="0.25">
+      <c r="D3"/>
+    </row>
+    <row r="4" spans="2:4" x14ac:dyDescent="0.25">
+      <c r="D4"/>
+    </row>
+    <row r="5" spans="2:4" x14ac:dyDescent="0.25">
+      <c r="D5"/>
+    </row>
+    <row r="6" spans="2:4" x14ac:dyDescent="0.25">
       <c r="B6" s="1"/>
       <c r="C6" s="1"/>
     </row>
-    <row r="7" spans="2:3" x14ac:dyDescent="0.25">
+    <row r="7" spans="2:4" x14ac:dyDescent="0.25">
       <c r="B7" s="1"/>
       <c r="C7" s="1"/>
     </row>
-    <row r="8" spans="2:3" x14ac:dyDescent="0.25">
+    <row r="8" spans="2:4" x14ac:dyDescent="0.25">
       <c r="B8" s="1"/>
       <c r="C8" s="1"/>
     </row>
-    <row r="9" spans="2:3" x14ac:dyDescent="0.25">
+    <row r="9" spans="2:4" x14ac:dyDescent="0.25">
       <c r="B9" s="1"/>
       <c r="C9" s="1"/>
     </row>
-    <row r="10" spans="2:3" x14ac:dyDescent="0.25">
+    <row r="10" spans="2:4" x14ac:dyDescent="0.25">
       <c r="B10" s="1"/>
       <c r="C10" s="1"/>
     </row>
-    <row r="11" spans="2:3" x14ac:dyDescent="0.25">
+    <row r="11" spans="2:4" x14ac:dyDescent="0.25">
       <c r="B11" s="1"/>
       <c r="C11" s="1"/>
     </row>
-    <row r="12" spans="2:3" x14ac:dyDescent="0.25">
+    <row r="12" spans="2:4" x14ac:dyDescent="0.25">
       <c r="B12" s="1"/>
       <c r="C12" s="1"/>
     </row>
-    <row r="13" spans="2:3" x14ac:dyDescent="0.25">
+    <row r="13" spans="2:4" x14ac:dyDescent="0.25">
       <c r="B13" s="1"/>
       <c r="C13" s="1"/>
     </row>
-    <row r="14" spans="2:3" x14ac:dyDescent="0.25">
+    <row r="14" spans="2:4" x14ac:dyDescent="0.25">
       <c r="B14" s="1"/>
       <c r="C14" s="1"/>
     </row>
-    <row r="15" spans="2:3" x14ac:dyDescent="0.25">
+    <row r="15" spans="2:4" x14ac:dyDescent="0.25">
       <c r="B15" s="1"/>
       <c r="C15" s="1"/>
     </row>
-    <row r="16" spans="2:3" x14ac:dyDescent="0.25">
+    <row r="16" spans="2:4" x14ac:dyDescent="0.25">
       <c r="B16" s="1"/>
       <c r="C16" s="1"/>
     </row>

</xml_diff>